<commit_message>
updated STOEND plotting function for UMAP
</commit_message>
<xml_diff>
--- a/Predictions/Validation/XY-Lipids_Predictions.xlsx
+++ b/Predictions/Validation/XY-Lipids_Predictions.xlsx
@@ -455,7 +455,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7421576976776123</v>
+        <v>0.7266183495521545</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6557300686836243</v>
+        <v>0.5818207859992981</v>
       </c>
     </row>
     <row r="4">
@@ -481,59 +481,59 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5495933294296265</v>
+        <v>0.5800464749336243</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OC(CN(CCCC)CCCC)(COCCCCCCCCCCCC)COCCCCCCCCCCCC</t>
+          <t>OC(CN(CC)CC)(COCCCCCCCCCCCC)COCCCCCCCCCCCC</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5471322536468506</v>
+        <v>0.553452730178833</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>OC(CN(CCCC)CCCC)(COC(CCCCC)=O)COC(CCCCC)=O</t>
+          <t>OC(CN(CCO)CCO)(COC(CCCCC)=O)COC(CCCCC)=O</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5083518028259277</v>
+        <v>0.5503665804862976</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>OC(CN(CCO)CCO)(COC(CCCCC)=O)COC(CCCCC)=O</t>
+          <t>OC(CN(CCCC)CCCC)(COC(CCCCC)=O)COC(CCCCC)=O</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5356972217559814</v>
+        <v>0.5457346439361572</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>OC(CN(CC)CC)(COCCCCCCCCCCCC)COCCCCCCCCCCCC</t>
+          <t>OC(CN(CCCC)CCCC)(COCCCCCCCCCCCC)COCCCCCCCCCCCC</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5180879831314087</v>
+        <v>0.5134831070899963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>